<commit_message>
completed 'draw lines' mini-test from Lab 3 instructions & added option to view inputs to microblaze from datapath's output slave registers
</commit_message>
<xml_diff>
--- a/Software_Controlled_Datapath/lab3_signal_mapping.xlsx
+++ b/Software_Controlled_Datapath/lab3_signal_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason.Wyche\source\repos\ece383_wksp\Software_Controlled_Datapath\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D376E07-28F6-4763-B5CD-2F842B42EDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A70EDF-98A1-4DBD-9B69-C21FDAC837E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="81">
   <si>
     <t>MicroBlaze Registers [in = read; out = write]</t>
   </si>
@@ -267,6 +267,18 @@
   </si>
   <si>
     <t>H17</t>
+  </si>
+  <si>
+    <t>switch(2)</t>
+  </si>
+  <si>
+    <t>switch(3)</t>
+  </si>
+  <si>
+    <t>switch(1)</t>
+  </si>
+  <si>
+    <t>switch(0)</t>
   </si>
 </sst>
 </file>
@@ -995,7 +1007,7 @@
         <v>45</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>73</v>
@@ -1006,7 +1018,7 @@
         <v>48</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>61</v>
@@ -1017,7 +1029,7 @@
         <v>51</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>75</v>
@@ -1028,7 +1040,7 @@
         <v>54</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>74</v>

</xml_diff>